<commit_message>
Renommage du dossier en Vertrauen et corrections+Style+ Vert & Graph1s with contrats1 + Taille2
</commit_message>
<xml_diff>
--- a/Dashbords/DB_Vertauren.xlsx
+++ b/Dashbords/DB_Vertauren.xlsx
@@ -8,12 +8,15 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\PC\Desktop\Project_2026\Vertrauen\Dashbords\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{487B1C4A-C0A0-47CE-9201-CCDD659F0DD7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{81314B62-2BC8-4490-86DA-6A8F73FA5CED}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{1E2A3A4A-D124-412E-945C-4FFB85A234FC}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{1E2A3A4A-D124-412E-945C-4FFB85A234FC}"/>
   </bookViews>
   <sheets>
-    <sheet name="Users" sheetId="1" r:id="rId1"/>
+    <sheet name="Unternehmen" sheetId="1" r:id="rId1"/>
+    <sheet name="Benutzer_Compagni" sheetId="2" r:id="rId2"/>
+    <sheet name="Angebote_Offre" sheetId="3" r:id="rId3"/>
+    <sheet name="Verträge_Contrat" sheetId="4" r:id="rId4"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -39,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11" uniqueCount="11">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="43" uniqueCount="32">
   <si>
     <t>created_at</t>
   </si>
@@ -72,16 +75,91 @@
   </si>
   <si>
     <t>Yassine</t>
+  </si>
+  <si>
+    <t>Mail</t>
+  </si>
+  <si>
+    <t>daoui00yassine@gmail.com</t>
+  </si>
+  <si>
+    <t>commercial</t>
+  </si>
+  <si>
+    <t>created</t>
+  </si>
+  <si>
+    <t>createdAt</t>
+  </si>
+  <si>
+    <t>name</t>
+  </si>
+  <si>
+    <t>phone</t>
+  </si>
+  <si>
+    <t>service</t>
+  </si>
+  <si>
+    <t>Elektrizität ,Gas</t>
+  </si>
+  <si>
+    <t>Youssef Daoui</t>
+  </si>
+  <si>
+    <r>
+      <t>Yello Strom</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="14"/>
+        <color rgb="FFFFFFFF"/>
+        <rFont val="Segoe UI"/>
+        <family val="2"/>
+      </rPr>
+      <t> </t>
+    </r>
+  </si>
+  <si>
+    <t>E WIE EINFACH</t>
+  </si>
+  <si>
+    <t>0221 789 658 00</t>
+  </si>
+  <si>
+    <t>Vattenfall</t>
+  </si>
+  <si>
+    <t>46 (0)8 739 50 00</t>
+  </si>
+  <si>
+    <t>EnBW Energie Baden-Württemberg AG</t>
+  </si>
+  <si>
+    <t xml:space="preserve">49 721 63-00 </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Rheinisch-Westfälisches Elektrizitätswerk </t>
+  </si>
+  <si>
+    <t>49 06026 - 4081771</t>
+  </si>
+  <si>
+    <t>1898-04-01</t>
+  </si>
+  <si>
+    <t xml:space="preserve">E-ON </t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="1">
-    <numFmt numFmtId="167" formatCode="[$-F800]dddd\,\ mmmm\ dd\,\ yyyy"/>
+  <numFmts count="2">
+    <numFmt numFmtId="164" formatCode="[$-F800]dddd\,\ mmmm\ dd\,\ yyyy"/>
+    <numFmt numFmtId="169" formatCode="0#&quot; &quot;##&quot; &quot;##&quot; &quot;##&quot; &quot;##"/>
   </numFmts>
-  <fonts count="3">
+  <fonts count="6">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -103,6 +181,27 @@
       <color theme="3" tint="9.9978637043366805E-2"/>
       <name val="Google Sans Code"/>
     </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="10"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="14"/>
+      <color rgb="FFFFFFFF"/>
+      <name val="Segoe UI"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="14"/>
+      <color theme="3" tint="9.9978637043366805E-2"/>
+      <name val="Segoe UI"/>
+      <family val="2"/>
+    </font>
   </fonts>
   <fills count="3">
     <fill>
@@ -118,7 +217,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="13">
+  <borders count="16">
     <border>
       <left/>
       <right/>
@@ -300,13 +399,51 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="23">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="167" fontId="1" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="1" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -345,8 +482,36 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="8" xfId="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="169" fontId="1" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="1" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Lien hypertexte" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -679,14 +844,17 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{72F4F883-F6DE-4039-807D-D7B2923163F6}">
-  <dimension ref="B1:H17"/>
+  <dimension ref="B1:I17"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4"/>
   <cols>
-    <col min="2" max="8" width="25.77734375" customWidth="1"/>
+    <col min="1" max="1" width="7.6640625" customWidth="1"/>
+    <col min="2" max="2" width="25.77734375" customWidth="1"/>
+    <col min="3" max="3" width="14.6640625" customWidth="1"/>
+    <col min="4" max="9" width="25.77734375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:8" ht="15" thickBot="1"/>
-    <row r="2" spans="2:8" ht="18" thickBot="1">
+    <row r="1" spans="2:9" ht="15" thickBot="1"/>
+    <row r="2" spans="2:9" ht="18" thickBot="1">
       <c r="B2" s="10" t="s">
         <v>0</v>
       </c>
@@ -694,169 +862,376 @@
         <v>1</v>
       </c>
       <c r="D2" s="11" t="s">
+        <v>11</v>
+      </c>
+      <c r="E2" s="11" t="s">
         <v>3</v>
       </c>
-      <c r="E2" s="11" t="s">
+      <c r="F2" s="11" t="s">
         <v>5</v>
       </c>
-      <c r="F2" s="11" t="s">
+      <c r="G2" s="11" t="s">
         <v>6</v>
       </c>
-      <c r="G2" s="11" t="s">
+      <c r="H2" s="11" t="s">
         <v>7</v>
       </c>
-      <c r="H2" s="12" t="s">
+      <c r="I2" s="12" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="3" spans="2:8">
+    <row r="3" spans="2:9">
       <c r="B3" s="1">
         <v>46241.764421296299</v>
       </c>
       <c r="C3" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="D3" s="2" t="s">
+      <c r="D3" s="14" t="s">
+        <v>12</v>
+      </c>
+      <c r="E3" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="E3" s="2" t="s">
+      <c r="F3" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="F3" s="2" t="s">
+      <c r="G3" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="G3" s="13">
+      <c r="H3" s="13">
         <v>21266694636</v>
       </c>
-      <c r="H3" s="3"/>
-    </row>
-    <row r="4" spans="2:8">
+      <c r="I3" s="3"/>
+    </row>
+    <row r="4" spans="2:9">
       <c r="B4" s="4"/>
       <c r="C4" s="5"/>
       <c r="D4" s="5"/>
       <c r="E4" s="5"/>
       <c r="F4" s="5"/>
       <c r="G4" s="5"/>
-      <c r="H4" s="6"/>
-    </row>
-    <row r="5" spans="2:8">
+      <c r="H4" s="5"/>
+      <c r="I4" s="6"/>
+    </row>
+    <row r="5" spans="2:9">
       <c r="B5" s="4"/>
       <c r="C5" s="5"/>
       <c r="D5" s="5"/>
       <c r="E5" s="5"/>
       <c r="F5" s="5"/>
       <c r="G5" s="5"/>
-      <c r="H5" s="6"/>
-    </row>
-    <row r="6" spans="2:8">
+      <c r="H5" s="5"/>
+      <c r="I5" s="6"/>
+    </row>
+    <row r="6" spans="2:9">
       <c r="B6" s="4"/>
       <c r="C6" s="5"/>
       <c r="D6" s="5"/>
       <c r="E6" s="5"/>
       <c r="F6" s="5"/>
       <c r="G6" s="5"/>
-      <c r="H6" s="6"/>
-    </row>
-    <row r="7" spans="2:8">
+      <c r="H6" s="5"/>
+      <c r="I6" s="6"/>
+    </row>
+    <row r="7" spans="2:9">
       <c r="B7" s="4"/>
       <c r="C7" s="5"/>
       <c r="D7" s="5"/>
       <c r="E7" s="5"/>
       <c r="F7" s="5"/>
       <c r="G7" s="5"/>
-      <c r="H7" s="6"/>
-    </row>
-    <row r="8" spans="2:8">
+      <c r="H7" s="5"/>
+      <c r="I7" s="6"/>
+    </row>
+    <row r="8" spans="2:9">
       <c r="B8" s="4"/>
       <c r="C8" s="5"/>
       <c r="D8" s="5"/>
       <c r="E8" s="5"/>
       <c r="F8" s="5"/>
       <c r="G8" s="5"/>
-      <c r="H8" s="6"/>
-    </row>
-    <row r="9" spans="2:8">
+      <c r="H8" s="5"/>
+      <c r="I8" s="6"/>
+    </row>
+    <row r="9" spans="2:9">
       <c r="B9" s="4"/>
       <c r="C9" s="5"/>
       <c r="D9" s="5"/>
       <c r="E9" s="5"/>
       <c r="F9" s="5"/>
       <c r="G9" s="5"/>
-      <c r="H9" s="6"/>
-    </row>
-    <row r="10" spans="2:8">
+      <c r="H9" s="5"/>
+      <c r="I9" s="6"/>
+    </row>
+    <row r="10" spans="2:9">
       <c r="B10" s="4"/>
       <c r="C10" s="5"/>
       <c r="D10" s="5"/>
       <c r="E10" s="5"/>
       <c r="F10" s="5"/>
       <c r="G10" s="5"/>
-      <c r="H10" s="6"/>
-    </row>
-    <row r="11" spans="2:8">
+      <c r="H10" s="5"/>
+      <c r="I10" s="6"/>
+    </row>
+    <row r="11" spans="2:9">
       <c r="B11" s="4"/>
       <c r="C11" s="5"/>
       <c r="D11" s="5"/>
       <c r="E11" s="5"/>
       <c r="F11" s="5"/>
       <c r="G11" s="5"/>
-      <c r="H11" s="6"/>
-    </row>
-    <row r="12" spans="2:8">
+      <c r="H11" s="5"/>
+      <c r="I11" s="6"/>
+    </row>
+    <row r="12" spans="2:9">
       <c r="B12" s="4"/>
       <c r="C12" s="5"/>
       <c r="D12" s="5"/>
       <c r="E12" s="5"/>
       <c r="F12" s="5"/>
       <c r="G12" s="5"/>
-      <c r="H12" s="6"/>
-    </row>
-    <row r="13" spans="2:8">
+      <c r="H12" s="5"/>
+      <c r="I12" s="6"/>
+    </row>
+    <row r="13" spans="2:9">
       <c r="B13" s="4"/>
       <c r="C13" s="5"/>
       <c r="D13" s="5"/>
       <c r="E13" s="5"/>
       <c r="F13" s="5"/>
       <c r="G13" s="5"/>
-      <c r="H13" s="6"/>
-    </row>
-    <row r="14" spans="2:8">
+      <c r="H13" s="5"/>
+      <c r="I13" s="6"/>
+    </row>
+    <row r="14" spans="2:9">
       <c r="B14" s="4"/>
       <c r="C14" s="5"/>
       <c r="D14" s="5"/>
       <c r="E14" s="5"/>
       <c r="F14" s="5"/>
       <c r="G14" s="5"/>
-      <c r="H14" s="6"/>
-    </row>
-    <row r="15" spans="2:8">
+      <c r="H14" s="5"/>
+      <c r="I14" s="6"/>
+    </row>
+    <row r="15" spans="2:9">
       <c r="B15" s="4"/>
       <c r="C15" s="5"/>
       <c r="D15" s="5"/>
       <c r="E15" s="5"/>
       <c r="F15" s="5"/>
       <c r="G15" s="5"/>
-      <c r="H15" s="6"/>
-    </row>
-    <row r="16" spans="2:8">
+      <c r="H15" s="5"/>
+      <c r="I15" s="6"/>
+    </row>
+    <row r="16" spans="2:9">
       <c r="B16" s="4"/>
       <c r="C16" s="5"/>
       <c r="D16" s="5"/>
       <c r="E16" s="5"/>
       <c r="F16" s="5"/>
       <c r="G16" s="5"/>
-      <c r="H16" s="6"/>
-    </row>
-    <row r="17" spans="2:8" ht="15" thickBot="1">
+      <c r="H16" s="5"/>
+      <c r="I16" s="6"/>
+    </row>
+    <row r="17" spans="2:9" ht="15" thickBot="1">
       <c r="B17" s="7"/>
       <c r="C17" s="8"/>
       <c r="D17" s="8"/>
       <c r="E17" s="8"/>
       <c r="F17" s="8"/>
       <c r="G17" s="8"/>
-      <c r="H17" s="9"/>
+      <c r="H17" s="8"/>
+      <c r="I17" s="9"/>
     </row>
   </sheetData>
+  <hyperlinks>
+    <hyperlink ref="D3" r:id="rId1" xr:uid="{16E0B3F4-577F-4290-9F1D-4D5B5FB7088F}"/>
+  </hyperlinks>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9C48D4EF-0DF8-4605-8763-893B33EDCE0E}">
+  <dimension ref="B1:G9"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4"/>
+  <cols>
+    <col min="1" max="1" width="11.5546875" style="17"/>
+    <col min="2" max="2" width="36.77734375" style="17" bestFit="1" customWidth="1"/>
+    <col min="3" max="7" width="18.6640625" style="17" customWidth="1"/>
+    <col min="8" max="16384" width="11.5546875" style="17"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="2:7" ht="15" thickBot="1"/>
+    <row r="2" spans="2:7" ht="21" thickBot="1">
+      <c r="B2" s="19" t="s">
+        <v>16</v>
+      </c>
+      <c r="C2" s="20" t="s">
+        <v>15</v>
+      </c>
+      <c r="D2" s="20" t="s">
+        <v>13</v>
+      </c>
+      <c r="E2" s="20" t="s">
+        <v>17</v>
+      </c>
+      <c r="F2" s="20" t="s">
+        <v>14</v>
+      </c>
+      <c r="G2" s="21" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="3" spans="2:7" ht="20.399999999999999">
+      <c r="B3" s="18" t="s">
+        <v>21</v>
+      </c>
+      <c r="C3" s="16">
+        <v>46235</v>
+      </c>
+      <c r="D3" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="E3" s="15">
+        <v>4922199690100</v>
+      </c>
+      <c r="F3" s="16">
+        <v>36192</v>
+      </c>
+      <c r="G3" s="3" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="4" spans="2:7">
+      <c r="B4" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="C4" s="16">
+        <v>46235</v>
+      </c>
+      <c r="D4" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="E4" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="F4" s="22">
+        <v>39114</v>
+      </c>
+      <c r="G4" s="3" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="5" spans="2:7">
+      <c r="B5" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="C5" s="16">
+        <v>46235</v>
+      </c>
+      <c r="D5" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="E5" s="5" t="s">
+        <v>25</v>
+      </c>
+      <c r="F5" s="22">
+        <v>3320</v>
+      </c>
+      <c r="G5" s="3" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="6" spans="2:7">
+      <c r="B6" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="C6" s="16">
+        <v>46235</v>
+      </c>
+      <c r="D6" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="E6" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="F6" s="22">
+        <v>35462</v>
+      </c>
+      <c r="G6" s="3" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="7" spans="2:7">
+      <c r="B7" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="C7" s="16">
+        <v>46235</v>
+      </c>
+      <c r="D7" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="E7" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="F7" s="5" t="s">
+        <v>30</v>
+      </c>
+      <c r="G7" s="3" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="8" spans="2:7">
+      <c r="B8" s="18" t="s">
+        <v>31</v>
+      </c>
+      <c r="C8" s="16">
+        <v>46235</v>
+      </c>
+      <c r="D8" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="E8" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="F8" s="16">
+        <v>36220</v>
+      </c>
+      <c r="G8" s="3" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="9" spans="2:7" ht="15" thickBot="1">
+      <c r="B9" s="7"/>
+      <c r="C9" s="8"/>
+      <c r="D9" s="8"/>
+      <c r="E9" s="8"/>
+      <c r="F9" s="8"/>
+      <c r="G9" s="9"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1E974358-5BD6-4E8B-B961-2C6A500DD9A0}">
+  <dimension ref="A1"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4"/>
+  <sheetData/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EDA15F77-33B7-4A9E-9FC2-544FBD24B1E7}">
+  <dimension ref="A1"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4"/>
+  <sheetData/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>